<commit_message>
fix(schema): keep in-toto's predicate key, which the adapt copy renames
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/in_toto_linkml.xlsx
+++ b/project/excel/in_toto_linkml.xlsx
@@ -1466,22 +1466,22 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>predicate</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>statement_type</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>subject</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>predicate_type</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>statement_predicate</t>
         </is>
       </c>
     </row>

</xml_diff>